<commit_message>
dedicated seeding override for Tractors 1 and 3
</commit_message>
<xml_diff>
--- a/seeding-efficiency-2026.xlsx
+++ b/seeding-efficiency-2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="101">
   <si>
     <t>Seeding Efficiency Report — 2026 Season</t>
   </si>
@@ -133,7 +133,7 @@
     <t>South</t>
   </si>
   <si>
-    <t>9RT 570 #20 UFER</t>
+    <t>8RT 370 #3 Ufer</t>
   </si>
   <si>
     <t>Borstad 19</t>
@@ -151,9 +151,6 @@
     <t>Butterfield SLM Quarter</t>
   </si>
   <si>
-    <t>8RT 370 #3 Ufer</t>
-  </si>
-  <si>
     <t>Dougs Qtr</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
     <t>Fancher 240</t>
   </si>
   <si>
-    <t>8RT 370 #3 Ufer, 9RT 570 #20 UFER</t>
-  </si>
-  <si>
     <t>Fancher North-North 131</t>
   </si>
   <si>
@@ -187,15 +181,12 @@
     <t>Greiner_Antrim Sec 20</t>
   </si>
   <si>
-    <t>865b Challenger</t>
+    <t>8RT 370 #3 Ufer, 865b Challenger</t>
   </si>
   <si>
     <t>Halverson Quarter</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8RT 370 #1 Ufer, 9620RX #21 UFER, 9RT 570 #20 UFER</t>
-  </si>
-  <si>
     <t>Hartman</t>
   </si>
   <si>
@@ -208,7 +199,7 @@
     <t>Home</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8RT 370 #1 Ufer, 8220T #6 Ufer, 9620RX #21 UFER, 9RT 570 #20 UFER</t>
+    <t>8220T #6 Ufer,  8RT 370 #1 Ufer</t>
   </si>
   <si>
     <t>Keithahn 190</t>
@@ -247,9 +238,6 @@
     <t>M-245 AGCO Jackson Embretson</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8RT 370 #1 Ufer, 9RT 570 #20 UFER, 9620RX #21 UFER</t>
-  </si>
-  <si>
     <t>M-256 Iverson Jackson Quarter</t>
   </si>
   <si>
@@ -262,15 +250,12 @@
     <t>Mau   230</t>
   </si>
   <si>
-    <t>8RT 370 #3 Ufer, 9620RX #21 UFER, 9RT 570 #20 UFER</t>
+    <t>8RT 370 #3 Ufer, 7250R Wheel #7 Ufer, 9620RX #21 UFER, 9RT 570 #20 UFER</t>
   </si>
   <si>
     <t>Niss  40</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8RT 370 #1 Ufer, 9620RX #21 UFER</t>
-  </si>
-  <si>
     <t>Ole Johnson North 80</t>
   </si>
   <si>
@@ -289,16 +274,10 @@
     <t>Rollof 80</t>
   </si>
   <si>
-    <t xml:space="preserve"> 8RT 370 #1 Ufer, 9RT 570 #20 UFER</t>
-  </si>
-  <si>
     <t>Schwanz 80</t>
   </si>
   <si>
     <t>Stradtman Home</t>
-  </si>
-  <si>
-    <t>8RT 370 #3 Ufer, 865b Challenger</t>
   </si>
   <si>
     <t>Stradtman Richards</t>
@@ -394,12 +373,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1A6A1A"/>
+      <color rgb="FF6B7A5A"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF6B7A5A"/>
+      <color rgb="FF1A6A1A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -505,16 +484,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -961,16 +940,16 @@
         <v>392.9</v>
       </c>
       <c r="F6" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" s="7">
-        <v>24</v>
+        <v>32.3</v>
       </c>
       <c r="H6" s="8">
-        <v>16.4</v>
+        <v>12.2</v>
       </c>
       <c r="I6" s="7">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>17</v>
@@ -1522,13 +1501,13 @@
         <v>1</v>
       </c>
       <c r="G24" s="11">
+        <v>7</v>
+      </c>
+      <c r="H24" s="15">
+        <v>29.8</v>
+      </c>
+      <c r="I24" s="11">
         <v>2</v>
-      </c>
-      <c r="H24" s="15">
-        <v>104.5</v>
-      </c>
-      <c r="I24" s="11">
-        <v>0.6</v>
       </c>
       <c r="J24" s="11" t="s">
         <v>40</v>
@@ -1627,12 +1606,12 @@
         <v>2</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>39</v>
@@ -1659,12 +1638,12 @@
         <v>1.9</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>39</v>
@@ -1691,12 +1670,12 @@
         <v>10.7</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>39</v>
@@ -1711,24 +1690,24 @@
         <v>210.08</v>
       </c>
       <c r="F30" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" s="11">
-        <v>9</v>
-      </c>
-      <c r="H30" s="19">
-        <v>23.3</v>
+        <v>6</v>
+      </c>
+      <c r="H30" s="11">
+        <v>35</v>
       </c>
       <c r="I30" s="11">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>39</v>
@@ -1755,12 +1734,12 @@
         <v>2.2</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>39</v>
@@ -1780,19 +1759,19 @@
       <c r="G32" s="11">
         <v>39.7</v>
       </c>
-      <c r="H32" s="19">
+      <c r="H32" s="15">
         <v>3.3</v>
       </c>
       <c r="I32" s="11">
         <v>18.2</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>39</v>
@@ -1819,12 +1798,12 @@
         <v>3.8</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>39</v>
@@ -1856,7 +1835,7 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>39</v>
@@ -1888,7 +1867,7 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>39</v>
@@ -1908,7 +1887,7 @@
       <c r="G36" s="11">
         <v>5.6</v>
       </c>
-      <c r="H36" s="19">
+      <c r="H36" s="15">
         <v>27.2</v>
       </c>
       <c r="I36" s="11">
@@ -1920,7 +1899,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>39</v>
@@ -1935,24 +1914,24 @@
         <v>78.36</v>
       </c>
       <c r="F37" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="7">
-        <v>2</v>
-      </c>
-      <c r="H37" s="7">
-        <v>39.2</v>
+        <v>4</v>
+      </c>
+      <c r="H37" s="8">
+        <v>19.5</v>
       </c>
       <c r="I37" s="7">
-        <v>1.5</v>
+        <v>3.1</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>39</v>
@@ -1967,24 +1946,24 @@
         <v>149.47</v>
       </c>
       <c r="F38" s="11">
+        <v>1</v>
+      </c>
+      <c r="G38" s="11">
         <v>3</v>
       </c>
-      <c r="G38" s="11">
-        <v>5</v>
-      </c>
-      <c r="H38" s="19">
-        <v>29.9</v>
+      <c r="H38" s="11">
+        <v>49.8</v>
       </c>
       <c r="I38" s="11">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>39</v>
@@ -2011,12 +1990,12 @@
         <v>3.9</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>39</v>
@@ -2036,19 +2015,19 @@
       <c r="G40" s="11">
         <v>5</v>
       </c>
-      <c r="H40" s="19">
+      <c r="H40" s="15">
         <v>21.2</v>
       </c>
       <c r="I40" s="11">
         <v>2.8</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>39</v>
@@ -2080,7 +2059,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>39</v>
@@ -2095,24 +2074,24 @@
         <v>215</v>
       </c>
       <c r="F42" s="11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G42" s="11">
-        <v>8.1</v>
-      </c>
-      <c r="H42" s="19">
-        <v>26.7</v>
+        <v>9</v>
+      </c>
+      <c r="H42" s="15">
+        <v>23.9</v>
       </c>
       <c r="I42" s="11">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>39</v>
@@ -2144,7 +2123,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>39</v>
@@ -2164,19 +2143,19 @@
       <c r="G44" s="11">
         <v>4</v>
       </c>
-      <c r="H44" s="19">
+      <c r="H44" s="15">
         <v>27.9</v>
       </c>
       <c r="I44" s="11">
         <v>2.2</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>39</v>
@@ -2203,12 +2182,12 @@
         <v>5.1</v>
       </c>
       <c r="J45" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>39</v>
@@ -2240,7 +2219,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>39</v>
@@ -2267,12 +2246,12 @@
         <v>1.6</v>
       </c>
       <c r="J47" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>39</v>
@@ -2292,7 +2271,7 @@
       <c r="G48" s="11">
         <v>8</v>
       </c>
-      <c r="H48" s="19">
+      <c r="H48" s="15">
         <v>14</v>
       </c>
       <c r="I48" s="11">
@@ -2304,7 +2283,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>39</v>
@@ -2336,7 +2315,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>39</v>
@@ -2368,7 +2347,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>39</v>
@@ -2400,7 +2379,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>39</v>
@@ -2432,7 +2411,7 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>39</v>
@@ -2452,7 +2431,7 @@
       <c r="G53" s="7">
         <v>3</v>
       </c>
-      <c r="H53" s="20">
+      <c r="H53" s="19">
         <v>51.6</v>
       </c>
       <c r="I53" s="7">
@@ -2464,7 +2443,7 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B54" s="9" t="s">
         <v>39</v>
@@ -2479,24 +2458,24 @@
         <v>185.91</v>
       </c>
       <c r="F54" s="11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G54" s="11">
-        <v>8.2</v>
-      </c>
-      <c r="H54" s="19">
-        <v>22.7</v>
+        <v>4.2</v>
+      </c>
+      <c r="H54" s="11">
+        <v>44.4</v>
       </c>
       <c r="I54" s="11">
-        <v>2.6</v>
+        <v>1.4</v>
       </c>
       <c r="J54" s="11" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>39</v>
@@ -2528,7 +2507,7 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B56" s="9" t="s">
         <v>39</v>
@@ -2548,19 +2527,19 @@
       <c r="G56" s="11">
         <v>3</v>
       </c>
-      <c r="H56" s="19">
+      <c r="H56" s="15">
         <v>12.3</v>
       </c>
       <c r="I56" s="11">
         <v>4.9</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>39</v>
@@ -2587,12 +2566,12 @@
         <v>1.8</v>
       </c>
       <c r="J57" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>39</v>
@@ -2607,24 +2586,24 @@
         <v>228.16</v>
       </c>
       <c r="F58" s="11">
+        <v>4</v>
+      </c>
+      <c r="G58" s="11">
+        <v>11.4</v>
+      </c>
+      <c r="H58" s="15">
+        <v>20</v>
+      </c>
+      <c r="I58" s="11">
         <v>3</v>
       </c>
-      <c r="G58" s="11">
-        <v>10.4</v>
-      </c>
-      <c r="H58" s="19">
-        <v>21.9</v>
-      </c>
-      <c r="I58" s="11">
-        <v>2.7</v>
-      </c>
       <c r="J58" s="11" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>39</v>
@@ -2639,24 +2618,24 @@
         <v>38.93</v>
       </c>
       <c r="F59" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G59" s="7">
-        <v>12.8</v>
-      </c>
-      <c r="H59" s="8">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="H59" s="7">
+        <v>38.9</v>
       </c>
       <c r="I59" s="7">
-        <v>20</v>
+        <v>1.5</v>
       </c>
       <c r="J59" s="7" t="s">
-        <v>85</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B60" s="9" t="s">
         <v>39</v>
@@ -2688,7 +2667,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>39</v>
@@ -2720,7 +2699,7 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B62" s="9" t="s">
         <v>39</v>
@@ -2752,7 +2731,7 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>39</v>
@@ -2784,7 +2763,7 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B64" s="9" t="s">
         <v>39</v>
@@ -2804,19 +2783,19 @@
       <c r="G64" s="11">
         <v>0.7</v>
       </c>
-      <c r="H64" s="15">
+      <c r="H64" s="20">
         <v>104.2</v>
       </c>
       <c r="I64" s="11">
         <v>0.6</v>
       </c>
       <c r="J64" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>39</v>
@@ -2831,24 +2810,24 @@
         <v>75.07</v>
       </c>
       <c r="F65" s="7">
+        <v>1</v>
+      </c>
+      <c r="G65" s="7">
         <v>2</v>
       </c>
-      <c r="G65" s="7">
-        <v>3</v>
-      </c>
-      <c r="H65" s="8">
-        <v>25</v>
+      <c r="H65" s="7">
+        <v>37.5</v>
       </c>
       <c r="I65" s="7">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="J65" s="7" t="s">
-        <v>92</v>
+        <v>42</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B66" s="9" t="s">
         <v>39</v>
@@ -2862,25 +2841,25 @@
       <c r="E66" s="11">
         <v>77.91</v>
       </c>
-      <c r="F66" s="11">
-        <v>1</v>
-      </c>
-      <c r="G66" s="11">
-        <v>1</v>
-      </c>
-      <c r="H66" s="15">
-        <v>77.9</v>
-      </c>
-      <c r="I66" s="11">
-        <v>0.8</v>
+      <c r="F66" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G66" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H66" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I66" s="11" t="s">
+        <v>19</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>39</v>
@@ -2907,12 +2886,12 @@
         <v>8</v>
       </c>
       <c r="J67" s="7" t="s">
-        <v>95</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B68" s="9" t="s">
         <v>39</v>
@@ -2944,7 +2923,7 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>39</v>
@@ -2976,7 +2955,7 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B70" s="9" t="s">
         <v>39</v>
@@ -2996,7 +2975,7 @@
       <c r="G70" s="11">
         <v>16.8</v>
       </c>
-      <c r="H70" s="19">
+      <c r="H70" s="15">
         <v>9</v>
       </c>
       <c r="I70" s="11">
@@ -3008,7 +2987,7 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>39</v>
@@ -3040,7 +3019,7 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B72" s="9" t="s">
         <v>39</v>
@@ -3067,12 +3046,12 @@
         <v>2</v>
       </c>
       <c r="J72" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>39</v>
@@ -3099,12 +3078,12 @@
         <v>4.7</v>
       </c>
       <c r="J73" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B74" s="9" t="s">
         <v>39</v>
@@ -3124,19 +3103,19 @@
       <c r="G74" s="11">
         <v>16.1</v>
       </c>
-      <c r="H74" s="19">
+      <c r="H74" s="15">
         <v>13.8</v>
       </c>
       <c r="I74" s="11">
         <v>4.3</v>
       </c>
       <c r="J74" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>39</v>
@@ -3168,7 +3147,7 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B76" s="9" t="s">
         <v>39</v>
@@ -3195,12 +3174,12 @@
         <v>1.6</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>39</v>
@@ -3220,19 +3199,19 @@
       <c r="G77" s="7">
         <v>1</v>
       </c>
-      <c r="H77" s="20">
+      <c r="H77" s="19">
         <v>64.1</v>
       </c>
       <c r="I77" s="7">
         <v>0.9</v>
       </c>
       <c r="J77" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="B78" s="9" t="s">
         <v>39</v>
@@ -3264,7 +3243,7 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="21" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B80" s="21" t="s">
         <v>19</v>
@@ -3279,13 +3258,13 @@
         <v>9698.489999999998</v>
       </c>
       <c r="F80" s="21">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G80" s="21">
-        <v>324.5</v>
+        <v>318.9</v>
       </c>
       <c r="H80" s="21">
-        <v>32.1</v>
+        <v>31</v>
       </c>
       <c r="I80" s="21" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
fixed cumulative GDUd on month, year, and weed views
</commit_message>
<xml_diff>
--- a/seeding-efficiency-2026.xlsx
+++ b/seeding-efficiency-2026.xlsx
@@ -22,7 +22,7 @@
     <t>Generated: Thursday, April 30, 2026</t>
   </si>
   <si>
-    <t>Fields with data: 45 of 72   |   Avg Ac/Hr: 32.4   |   Total Planter Hrs: 275.3   |   Source: Planter GPS</t>
+    <t>Fields with data: 45 of 72   |   Avg Ac/Hr: 39.7   |   Total Planter Hrs: 254.3   |   Source: Planter GPS</t>
   </si>
   <si>
     <t>Field</t>
@@ -397,22 +397,22 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="FFAA7700"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b/>
       <color rgb="FF5A6A4A"/>
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="FFAA7700"/>
+      <b/>
+      <color rgb="FF1A7A1A"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
       <color rgb="FFCC3300"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1A7A1A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -570,7 +570,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -586,24 +586,24 @@
     <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1522,16 +1522,16 @@
         <v>208.92</v>
       </c>
       <c r="F25" s="19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" s="15">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="H25" s="20">
-        <v>52.2</v>
+        <v>38.7</v>
       </c>
       <c r="I25" s="21">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="J25" s="13" t="s">
         <v>41</v>
@@ -1614,13 +1614,13 @@
         <v>1</v>
       </c>
       <c r="G28" s="9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H28" s="27">
-        <v>29.6</v>
+        <v>147.9</v>
       </c>
       <c r="I28" s="25">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>41</v>
@@ -1648,7 +1648,7 @@
       <c r="G29" s="15">
         <v>5</v>
       </c>
-      <c r="H29" s="28">
+      <c r="H29" s="20">
         <v>31</v>
       </c>
       <c r="I29" s="21">
@@ -1668,23 +1668,23 @@
       <c r="C30" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E30" s="9">
         <v>108.84</v>
       </c>
       <c r="F30" s="23">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G30" s="9">
-        <v>19.32</v>
-      </c>
-      <c r="H30" s="30">
-        <v>5.6</v>
+        <v>20.88</v>
+      </c>
+      <c r="H30" s="29">
+        <v>5.2</v>
       </c>
       <c r="I30" s="25">
-        <v>10.6</v>
+        <v>11.5</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>41</v>
@@ -1710,13 +1710,13 @@
         <v>1</v>
       </c>
       <c r="G31" s="15">
-        <v>6</v>
-      </c>
-      <c r="H31" s="28">
-        <v>35</v>
+        <v>6.9</v>
+      </c>
+      <c r="H31" s="20">
+        <v>30.4</v>
       </c>
       <c r="I31" s="21">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="J31" s="13" t="s">
         <v>41</v>
@@ -1732,7 +1732,7 @@
       <c r="C32" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="D32" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E32" s="9">
@@ -1742,13 +1742,13 @@
         <v>1</v>
       </c>
       <c r="G32" s="9">
-        <v>4.73</v>
+        <v>0.72</v>
       </c>
       <c r="H32" s="27">
-        <v>27.1</v>
+        <v>179</v>
       </c>
       <c r="I32" s="25">
-        <v>2.2</v>
+        <v>0.3</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>41</v>
@@ -1771,16 +1771,16 @@
         <v>132.11</v>
       </c>
       <c r="F33" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="15">
-        <v>41.7</v>
-      </c>
-      <c r="H33" s="31">
-        <v>3.2</v>
+        <v>5.67</v>
+      </c>
+      <c r="H33" s="30">
+        <v>23.3</v>
       </c>
       <c r="I33" s="21">
-        <v>18.9</v>
+        <v>2.6</v>
       </c>
       <c r="J33" s="13" t="s">
         <v>41</v>
@@ -1796,7 +1796,7 @@
       <c r="C34" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="D34" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="9">
@@ -1808,7 +1808,7 @@
       <c r="G34" s="9">
         <v>3</v>
       </c>
-      <c r="H34" s="30">
+      <c r="H34" s="29">
         <v>15.6</v>
       </c>
       <c r="I34" s="25">
@@ -1840,7 +1840,7 @@
       <c r="G35" s="15">
         <v>1</v>
       </c>
-      <c r="H35" s="20">
+      <c r="H35" s="31">
         <v>42.1</v>
       </c>
       <c r="I35" s="21">
@@ -1961,7 +1961,7 @@
       <c r="G39" s="15">
         <v>3</v>
       </c>
-      <c r="H39" s="20">
+      <c r="H39" s="31">
         <v>49.8</v>
       </c>
       <c r="I39" s="21">
@@ -1981,23 +1981,23 @@
       <c r="C40" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D40" s="29" t="s">
+      <c r="D40" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E40" s="9">
         <v>73.6</v>
       </c>
       <c r="F40" s="23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G40" s="9">
-        <v>4.48</v>
-      </c>
-      <c r="H40" s="30">
-        <v>16.4</v>
+        <v>6.5</v>
+      </c>
+      <c r="H40" s="29">
+        <v>11.3</v>
       </c>
       <c r="I40" s="25">
-        <v>3.7</v>
+        <v>5.3</v>
       </c>
       <c r="J40" s="7" t="s">
         <v>41</v>
@@ -2025,7 +2025,7 @@
       <c r="G41" s="15">
         <v>5</v>
       </c>
-      <c r="H41" s="31">
+      <c r="H41" s="30">
         <v>21.2</v>
       </c>
       <c r="I41" s="21">
@@ -2045,7 +2045,7 @@
       <c r="C42" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D42" s="29" t="s">
+      <c r="D42" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E42" s="9">
@@ -2080,13 +2080,13 @@
         <v>1</v>
       </c>
       <c r="G43" s="15">
-        <v>5</v>
-      </c>
-      <c r="H43" s="20">
-        <v>43</v>
+        <v>5.32</v>
+      </c>
+      <c r="H43" s="31">
+        <v>40.4</v>
       </c>
       <c r="I43" s="21">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="J43" s="13" t="s">
         <v>43</v>
@@ -2134,16 +2134,16 @@
         <v>111.48</v>
       </c>
       <c r="F45" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="15">
-        <v>4.48</v>
-      </c>
-      <c r="H45" s="31">
-        <v>24.9</v>
+        <v>4.97</v>
+      </c>
+      <c r="H45" s="30">
+        <v>22.4</v>
       </c>
       <c r="I45" s="21">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="J45" s="13" t="s">
         <v>41</v>
@@ -2166,16 +2166,16 @@
         <v>149.41</v>
       </c>
       <c r="F46" s="23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G46" s="9">
-        <v>12.72</v>
-      </c>
-      <c r="H46" s="30">
-        <v>11.7</v>
+        <v>18.23</v>
+      </c>
+      <c r="H46" s="29">
+        <v>8.2</v>
       </c>
       <c r="I46" s="25">
-        <v>5.1</v>
+        <v>7.3</v>
       </c>
       <c r="J46" s="7" t="s">
         <v>41</v>
@@ -2228,7 +2228,7 @@
       <c r="G48" s="9">
         <v>2</v>
       </c>
-      <c r="H48" s="27">
+      <c r="H48" s="33">
         <v>37.9</v>
       </c>
       <c r="I48" s="25">
@@ -2255,16 +2255,16 @@
         <v>111.89</v>
       </c>
       <c r="F49" s="19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G49" s="15">
-        <v>8.85</v>
-      </c>
-      <c r="H49" s="31">
-        <v>12.6</v>
+        <v>9.6</v>
+      </c>
+      <c r="H49" s="30">
+        <v>11.7</v>
       </c>
       <c r="I49" s="21">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="J49" s="13" t="s">
         <v>43</v>
@@ -2292,7 +2292,7 @@
       <c r="G50" s="9">
         <v>4</v>
       </c>
-      <c r="H50" s="27">
+      <c r="H50" s="33">
         <v>39.2</v>
       </c>
       <c r="I50" s="25">
@@ -2347,7 +2347,7 @@
       <c r="G52" s="9">
         <v>4.23</v>
       </c>
-      <c r="H52" s="27">
+      <c r="H52" s="33">
         <v>33.3</v>
       </c>
       <c r="I52" s="25">
@@ -2379,7 +2379,7 @@
       <c r="G53" s="15">
         <v>5</v>
       </c>
-      <c r="H53" s="28">
+      <c r="H53" s="20">
         <v>38.6</v>
       </c>
       <c r="I53" s="21">
@@ -2409,13 +2409,13 @@
         <v>1</v>
       </c>
       <c r="G54" s="9">
-        <v>4.43</v>
+        <v>1.28</v>
       </c>
       <c r="H54" s="27">
-        <v>34.9</v>
+        <v>120.6</v>
       </c>
       <c r="I54" s="25">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="J54" s="7" t="s">
         <v>43</v>
@@ -2438,16 +2438,16 @@
         <v>185.91</v>
       </c>
       <c r="F55" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G55" s="15">
-        <v>4.43</v>
-      </c>
-      <c r="H55" s="20">
-        <v>41.9</v>
+        <v>3.42</v>
+      </c>
+      <c r="H55" s="31">
+        <v>54.4</v>
       </c>
       <c r="I55" s="21">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="J55" s="13" t="s">
         <v>43</v>
@@ -2470,16 +2470,16 @@
         <v>147.73</v>
       </c>
       <c r="F56" s="23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G56" s="9">
-        <v>4.18</v>
-      </c>
-      <c r="H56" s="27">
-        <v>35.3</v>
+        <v>3.18</v>
+      </c>
+      <c r="H56" s="24">
+        <v>46.4</v>
       </c>
       <c r="I56" s="25">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="J56" s="7" t="s">
         <v>43</v>
@@ -2507,7 +2507,7 @@
       <c r="G57" s="15">
         <v>3</v>
       </c>
-      <c r="H57" s="31">
+      <c r="H57" s="30">
         <v>12.3</v>
       </c>
       <c r="I57" s="21">
@@ -2539,7 +2539,7 @@
       <c r="G58" s="9">
         <v>2</v>
       </c>
-      <c r="H58" s="27">
+      <c r="H58" s="33">
         <v>34.1</v>
       </c>
       <c r="I58" s="25">
@@ -2571,7 +2571,7 @@
       <c r="G59" s="15">
         <v>8</v>
       </c>
-      <c r="H59" s="28">
+      <c r="H59" s="20">
         <v>28.5</v>
       </c>
       <c r="I59" s="21">
@@ -2603,7 +2603,7 @@
       <c r="G60" s="9">
         <v>1</v>
       </c>
-      <c r="H60" s="27">
+      <c r="H60" s="33">
         <v>38.9</v>
       </c>
       <c r="I60" s="25">
@@ -2685,7 +2685,7 @@
       <c r="G63" s="15">
         <v>3</v>
       </c>
-      <c r="H63" s="20">
+      <c r="H63" s="31">
         <v>49.7</v>
       </c>
       <c r="I63" s="21">
@@ -2705,7 +2705,7 @@
       <c r="C64" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D64" s="29" t="s">
+      <c r="D64" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E64" s="9">
@@ -2717,7 +2717,7 @@
       <c r="G64" s="9">
         <v>4</v>
       </c>
-      <c r="H64" s="27">
+      <c r="H64" s="33">
         <v>34.3</v>
       </c>
       <c r="I64" s="25">
@@ -2749,7 +2749,7 @@
       <c r="G65" s="15">
         <v>1.53</v>
       </c>
-      <c r="H65" s="20">
+      <c r="H65" s="31">
         <v>49.8</v>
       </c>
       <c r="I65" s="21">
@@ -2769,7 +2769,7 @@
       <c r="C66" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D66" s="29" t="s">
+      <c r="D66" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E66" s="9">
@@ -2781,7 +2781,7 @@
       <c r="G66" s="9">
         <v>2</v>
       </c>
-      <c r="H66" s="27">
+      <c r="H66" s="33">
         <v>37.5</v>
       </c>
       <c r="I66" s="25">
@@ -2833,16 +2833,16 @@
         <v>172.03</v>
       </c>
       <c r="F68" s="23">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G68" s="9">
-        <v>20.73</v>
-      </c>
-      <c r="H68" s="30">
-        <v>8.3</v>
+        <v>26.67</v>
+      </c>
+      <c r="H68" s="29">
+        <v>6.5</v>
       </c>
       <c r="I68" s="25">
-        <v>7.2</v>
+        <v>9.3</v>
       </c>
       <c r="J68" s="7" t="s">
         <v>41</v>
@@ -2870,7 +2870,7 @@
       <c r="G69" s="15">
         <v>3</v>
       </c>
-      <c r="H69" s="20">
+      <c r="H69" s="31">
         <v>43.3</v>
       </c>
       <c r="I69" s="21">
@@ -2890,23 +2890,23 @@
       <c r="C70" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D70" s="29" t="s">
+      <c r="D70" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E70" s="9">
         <v>149.61</v>
       </c>
       <c r="F70" s="23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G70" s="9">
-        <v>3.65</v>
-      </c>
-      <c r="H70" s="24">
-        <v>41</v>
+        <v>4.3</v>
+      </c>
+      <c r="H70" s="33">
+        <v>34.8</v>
       </c>
       <c r="I70" s="25">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="J70" s="7" t="s">
         <v>43</v>
@@ -2929,16 +2929,16 @@
         <v>151.47</v>
       </c>
       <c r="F71" s="19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G71" s="15">
-        <v>16.78</v>
-      </c>
-      <c r="H71" s="31">
-        <v>9</v>
+        <v>19.45</v>
+      </c>
+      <c r="H71" s="30">
+        <v>7.8</v>
       </c>
       <c r="I71" s="21">
-        <v>6.6</v>
+        <v>7.7</v>
       </c>
       <c r="J71" s="13" t="s">
         <v>43</v>
@@ -2954,23 +2954,23 @@
       <c r="C72" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D72" s="29" t="s">
+      <c r="D72" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E72" s="9">
         <v>71.68</v>
       </c>
       <c r="F72" s="23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" s="9">
-        <v>2</v>
-      </c>
-      <c r="H72" s="27">
-        <v>35.8</v>
+        <v>2.8</v>
+      </c>
+      <c r="H72" s="33">
+        <v>25.6</v>
       </c>
       <c r="I72" s="25">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="J72" s="7" t="s">
         <v>43</v>
@@ -2998,7 +2998,7 @@
       <c r="G73" s="15">
         <v>2</v>
       </c>
-      <c r="H73" s="28">
+      <c r="H73" s="20">
         <v>30.3</v>
       </c>
       <c r="I73" s="21">
@@ -3018,23 +3018,23 @@
       <c r="C74" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D74" s="29" t="s">
+      <c r="D74" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E74" s="9">
         <v>136.86</v>
       </c>
       <c r="F74" s="23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G74" s="9">
-        <v>10.93</v>
-      </c>
-      <c r="H74" s="30">
-        <v>12.5</v>
+        <v>11.93</v>
+      </c>
+      <c r="H74" s="29">
+        <v>11.5</v>
       </c>
       <c r="I74" s="25">
-        <v>4.8</v>
+        <v>5.2</v>
       </c>
       <c r="J74" s="7" t="s">
         <v>41</v>
@@ -3057,16 +3057,16 @@
         <v>221.85</v>
       </c>
       <c r="F75" s="19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G75" s="15">
-        <v>16.12</v>
-      </c>
-      <c r="H75" s="31">
-        <v>13.8</v>
+        <v>16.85</v>
+      </c>
+      <c r="H75" s="30">
+        <v>13.2</v>
       </c>
       <c r="I75" s="21">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="J75" s="13" t="s">
         <v>41</v>
@@ -3082,7 +3082,7 @@
       <c r="C76" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D76" s="29" t="s">
+      <c r="D76" s="28" t="s">
         <v>45</v>
       </c>
       <c r="E76" s="9">
@@ -3114,16 +3114,16 @@
         <v>76.06</v>
       </c>
       <c r="F77" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G77" s="15">
-        <v>3.3</v>
-      </c>
-      <c r="H77" s="31">
-        <v>23</v>
+        <v>6.17</v>
+      </c>
+      <c r="H77" s="30">
+        <v>12.3</v>
       </c>
       <c r="I77" s="21">
-        <v>2.6</v>
+        <v>4.9</v>
       </c>
       <c r="J77" s="13" t="s">
         <v>41</v>
@@ -3151,7 +3151,7 @@
       <c r="G78" s="9">
         <v>1</v>
       </c>
-      <c r="H78" s="33">
+      <c r="H78" s="27">
         <v>64.1</v>
       </c>
       <c r="I78" s="25">
@@ -3178,16 +3178,16 @@
         <v>130.97</v>
       </c>
       <c r="F79" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" s="15">
-        <v>3.55</v>
-      </c>
-      <c r="H79" s="28">
-        <v>36.9</v>
+        <v>4.1</v>
+      </c>
+      <c r="H79" s="20">
+        <v>31.9</v>
       </c>
       <c r="I79" s="21">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="J79" s="13" t="s">
         <v>43</v>
@@ -3210,16 +3210,16 @@
         <v>9698.489999999998</v>
       </c>
       <c r="F81" s="36">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="G81" s="35">
-        <v>275.32</v>
+        <v>254.28</v>
       </c>
       <c r="H81" s="37">
-        <v>32.4</v>
+        <v>39.7</v>
       </c>
       <c r="I81" s="37">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="J81" s="34" t="s">
         <v>99</v>

</xml_diff>